<commit_message>
chore: update gitignore to ignore root generated reports and cache directories
</commit_message>
<xml_diff>
--- a/qa/reports/FARMAI_QA_300_Test_Cases.xlsx
+++ b/qa/reports/FARMAI_QA_300_Test_Cases.xlsx
@@ -27310,7 +27310,7 @@
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
@@ -27405,7 +27405,7 @@
       </c>
       <c r="L3" s="10" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M3" s="10" t="inlineStr">
@@ -27500,7 +27500,7 @@
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
@@ -27595,7 +27595,7 @@
       </c>
       <c r="L5" s="10" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M5" s="10" t="inlineStr">
@@ -27690,7 +27690,7 @@
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
@@ -27785,7 +27785,7 @@
       </c>
       <c r="L7" s="10" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M7" s="10" t="inlineStr">
@@ -27880,7 +27880,7 @@
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
@@ -27975,7 +27975,7 @@
       </c>
       <c r="L9" s="10" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M9" s="10" t="inlineStr">
@@ -28070,7 +28070,7 @@
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
@@ -28165,7 +28165,7 @@
       </c>
       <c r="L11" s="10" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M11" s="10" t="inlineStr">
@@ -28260,7 +28260,7 @@
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M12" s="3" t="inlineStr">
@@ -28355,7 +28355,7 @@
       </c>
       <c r="L13" s="10" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M13" s="10" t="inlineStr">
@@ -28450,7 +28450,7 @@
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr">
@@ -28545,7 +28545,7 @@
       </c>
       <c r="L15" s="10" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M15" s="10" t="inlineStr">
@@ -28640,7 +28640,7 @@
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr">
@@ -28735,7 +28735,7 @@
       </c>
       <c r="L17" s="10" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M17" s="10" t="inlineStr">
@@ -28830,7 +28830,7 @@
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr">
@@ -28925,7 +28925,7 @@
       </c>
       <c r="L19" s="10" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M19" s="10" t="inlineStr">
@@ -29020,7 +29020,7 @@
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M20" s="3" t="inlineStr">
@@ -29115,7 +29115,7 @@
       </c>
       <c r="L21" s="10" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M21" s="10" t="inlineStr">
@@ -29210,7 +29210,7 @@
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M22" s="3" t="inlineStr">
@@ -29305,7 +29305,7 @@
       </c>
       <c r="L23" s="10" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M23" s="10" t="inlineStr">
@@ -29400,7 +29400,7 @@
       </c>
       <c r="L24" s="3" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M24" s="3" t="inlineStr">
@@ -29495,7 +29495,7 @@
       </c>
       <c r="L25" s="10" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M25" s="10" t="inlineStr">
@@ -29590,7 +29590,7 @@
       </c>
       <c r="L26" s="3" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M26" s="3" t="inlineStr">
@@ -29685,7 +29685,7 @@
       </c>
       <c r="L27" s="10" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M27" s="10" t="inlineStr">
@@ -29780,7 +29780,7 @@
       </c>
       <c r="L28" s="3" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M28" s="3" t="inlineStr">
@@ -29875,7 +29875,7 @@
       </c>
       <c r="L29" s="10" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M29" s="10" t="inlineStr">
@@ -29970,7 +29970,7 @@
       </c>
       <c r="L30" s="3" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M30" s="3" t="inlineStr">
@@ -30065,7 +30065,7 @@
       </c>
       <c r="L31" s="10" t="inlineStr">
         <is>
-          <t>08:26:01</t>
+          <t>12:34:49</t>
         </is>
       </c>
       <c r="M31" s="10" t="inlineStr">

</xml_diff>

<commit_message>
style: redesign image uploaders to compact OneUI style and add leaf/pest file name validation filters
</commit_message>
<xml_diff>
--- a/qa/reports/FARMAI_QA_300_Test_Cases.xlsx
+++ b/qa/reports/FARMAI_QA_300_Test_Cases.xlsx
@@ -27310,7 +27310,7 @@
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
@@ -27405,7 +27405,7 @@
       </c>
       <c r="L3" s="10" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M3" s="10" t="inlineStr">
@@ -27500,7 +27500,7 @@
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
@@ -27595,7 +27595,7 @@
       </c>
       <c r="L5" s="10" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M5" s="10" t="inlineStr">
@@ -27690,7 +27690,7 @@
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
@@ -27785,7 +27785,7 @@
       </c>
       <c r="L7" s="10" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M7" s="10" t="inlineStr">
@@ -27880,7 +27880,7 @@
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
@@ -27975,7 +27975,7 @@
       </c>
       <c r="L9" s="10" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M9" s="10" t="inlineStr">
@@ -28070,7 +28070,7 @@
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
@@ -28165,7 +28165,7 @@
       </c>
       <c r="L11" s="10" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M11" s="10" t="inlineStr">
@@ -28260,7 +28260,7 @@
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M12" s="3" t="inlineStr">
@@ -28355,7 +28355,7 @@
       </c>
       <c r="L13" s="10" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M13" s="10" t="inlineStr">
@@ -28450,7 +28450,7 @@
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr">
@@ -28545,7 +28545,7 @@
       </c>
       <c r="L15" s="10" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M15" s="10" t="inlineStr">
@@ -28640,7 +28640,7 @@
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr">
@@ -28735,7 +28735,7 @@
       </c>
       <c r="L17" s="10" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M17" s="10" t="inlineStr">
@@ -28830,7 +28830,7 @@
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr">
@@ -28925,7 +28925,7 @@
       </c>
       <c r="L19" s="10" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M19" s="10" t="inlineStr">
@@ -29020,7 +29020,7 @@
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M20" s="3" t="inlineStr">
@@ -29115,7 +29115,7 @@
       </c>
       <c r="L21" s="10" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M21" s="10" t="inlineStr">
@@ -29210,7 +29210,7 @@
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M22" s="3" t="inlineStr">
@@ -29305,7 +29305,7 @@
       </c>
       <c r="L23" s="10" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M23" s="10" t="inlineStr">
@@ -29400,7 +29400,7 @@
       </c>
       <c r="L24" s="3" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M24" s="3" t="inlineStr">
@@ -29495,7 +29495,7 @@
       </c>
       <c r="L25" s="10" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M25" s="10" t="inlineStr">
@@ -29590,7 +29590,7 @@
       </c>
       <c r="L26" s="3" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M26" s="3" t="inlineStr">
@@ -29685,7 +29685,7 @@
       </c>
       <c r="L27" s="10" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M27" s="10" t="inlineStr">
@@ -29780,7 +29780,7 @@
       </c>
       <c r="L28" s="3" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M28" s="3" t="inlineStr">
@@ -29875,7 +29875,7 @@
       </c>
       <c r="L29" s="10" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M29" s="10" t="inlineStr">
@@ -29970,7 +29970,7 @@
       </c>
       <c r="L30" s="3" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M30" s="3" t="inlineStr">
@@ -30065,7 +30065,7 @@
       </c>
       <c r="L31" s="10" t="inlineStr">
         <is>
-          <t>12:34:49</t>
+          <t>14:24:48</t>
         </is>
       </c>
       <c r="M31" s="10" t="inlineStr">

</xml_diff>

<commit_message>
feat: integrate TensorFlow Lite image classification for crop leaf disease detection with Android & Web compatibility
</commit_message>
<xml_diff>
--- a/qa/reports/FARMAI_QA_300_Test_Cases.xlsx
+++ b/qa/reports/FARMAI_QA_300_Test_Cases.xlsx
@@ -27310,7 +27310,7 @@
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
@@ -27405,7 +27405,7 @@
       </c>
       <c r="L3" s="10" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M3" s="10" t="inlineStr">
@@ -27500,7 +27500,7 @@
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
@@ -27595,7 +27595,7 @@
       </c>
       <c r="L5" s="10" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M5" s="10" t="inlineStr">
@@ -27690,7 +27690,7 @@
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
@@ -27785,7 +27785,7 @@
       </c>
       <c r="L7" s="10" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M7" s="10" t="inlineStr">
@@ -27880,7 +27880,7 @@
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
@@ -27975,7 +27975,7 @@
       </c>
       <c r="L9" s="10" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M9" s="10" t="inlineStr">
@@ -28070,7 +28070,7 @@
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
@@ -28165,7 +28165,7 @@
       </c>
       <c r="L11" s="10" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M11" s="10" t="inlineStr">
@@ -28260,7 +28260,7 @@
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M12" s="3" t="inlineStr">
@@ -28355,7 +28355,7 @@
       </c>
       <c r="L13" s="10" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M13" s="10" t="inlineStr">
@@ -28450,7 +28450,7 @@
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr">
@@ -28545,7 +28545,7 @@
       </c>
       <c r="L15" s="10" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M15" s="10" t="inlineStr">
@@ -28640,7 +28640,7 @@
       </c>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr">
@@ -28735,7 +28735,7 @@
       </c>
       <c r="L17" s="10" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M17" s="10" t="inlineStr">
@@ -28830,7 +28830,7 @@
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr">
@@ -28925,7 +28925,7 @@
       </c>
       <c r="L19" s="10" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M19" s="10" t="inlineStr">
@@ -29020,7 +29020,7 @@
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M20" s="3" t="inlineStr">
@@ -29115,7 +29115,7 @@
       </c>
       <c r="L21" s="10" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M21" s="10" t="inlineStr">
@@ -29210,7 +29210,7 @@
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M22" s="3" t="inlineStr">
@@ -29305,7 +29305,7 @@
       </c>
       <c r="L23" s="10" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M23" s="10" t="inlineStr">
@@ -29400,7 +29400,7 @@
       </c>
       <c r="L24" s="3" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M24" s="3" t="inlineStr">
@@ -29495,7 +29495,7 @@
       </c>
       <c r="L25" s="10" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M25" s="10" t="inlineStr">
@@ -29590,7 +29590,7 @@
       </c>
       <c r="L26" s="3" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M26" s="3" t="inlineStr">
@@ -29685,7 +29685,7 @@
       </c>
       <c r="L27" s="10" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M27" s="10" t="inlineStr">
@@ -29780,7 +29780,7 @@
       </c>
       <c r="L28" s="3" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M28" s="3" t="inlineStr">
@@ -29875,7 +29875,7 @@
       </c>
       <c r="L29" s="10" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M29" s="10" t="inlineStr">
@@ -29970,7 +29970,7 @@
       </c>
       <c r="L30" s="3" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M30" s="3" t="inlineStr">
@@ -30065,7 +30065,7 @@
       </c>
       <c r="L31" s="10" t="inlineStr">
         <is>
-          <t>14:24:48</t>
+          <t>14:56:52</t>
         </is>
       </c>
       <c r="M31" s="10" t="inlineStr">

</xml_diff>